<commit_message>
Separate faulty AI extractions
</commit_message>
<xml_diff>
--- a/data/AI extractions/manifest.xlsx
+++ b/data/AI extractions/manifest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest" sheetId="1" r:id="R7832b988ecc948de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest" sheetId="1" r:id="Ra83f2d92ff794a53"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -417,13 +417,13 @@
         <x:v>../references/sps_references_export.ris#record-4</x:v>
       </x:c>
       <x:c r="G3" s="11" t="str">
-        <x:v>deepseek/17.json</x:v>
+        <x:v>faulty/deepseek/17.json</x:v>
       </x:c>
       <x:c r="H3" s="11" t="str">
-        <x:v>nemotron/17.json</x:v>
+        <x:v>faulty/nemotron/17.json</x:v>
       </x:c>
       <x:c r="I3" s="11" t="str">
-        <x:v>glm/17.json</x:v>
+        <x:v>faulty/glm/17.json</x:v>
       </x:c>
       <x:c r="J3" s="10" t="n">
         <x:f>COUNTA(G3:I3)</x:f>
@@ -499,13 +499,13 @@
         <x:v>../references/sps_references_export.ris#record-12</x:v>
       </x:c>
       <x:c r="G5" s="11" t="str">
-        <x:v>deepseek/38.json</x:v>
+        <x:v>faulty/deepseek/38.json</x:v>
       </x:c>
       <x:c r="H5" s="11" t="str">
-        <x:v>nemotron/38.json</x:v>
+        <x:v>faulty/nemotron/38.json</x:v>
       </x:c>
       <x:c r="I5" s="11" t="str">
-        <x:v>glm/38.json</x:v>
+        <x:v>faulty/glm/38.json</x:v>
       </x:c>
       <x:c r="J5" s="10" t="n">
         <x:f>COUNTA(G5:I5)</x:f>
@@ -704,13 +704,13 @@
         <x:v>../references/sps_references_export.ris#record-26</x:v>
       </x:c>
       <x:c r="G10" s="11" t="str">
-        <x:v>deepseek/85.json</x:v>
+        <x:v>faulty/deepseek/85.json</x:v>
       </x:c>
       <x:c r="H10" s="11" t="str">
-        <x:v>nemotron/85.json</x:v>
+        <x:v>faulty/nemotron/85.json</x:v>
       </x:c>
       <x:c r="I10" s="11" t="str">
-        <x:v>glm/85.json</x:v>
+        <x:v>faulty/glm/85.json</x:v>
       </x:c>
       <x:c r="J10" s="10" t="n">
         <x:f>COUNTA(G10:I10)</x:f>
@@ -786,13 +786,13 @@
         <x:v>../references/sps_references_export.ris#record-31</x:v>
       </x:c>
       <x:c r="G12" s="11" t="str">
-        <x:v>deepseek/101.json</x:v>
+        <x:v>faulty/deepseek/101.json</x:v>
       </x:c>
       <x:c r="H12" s="11" t="str">
-        <x:v>nemotron/101.json</x:v>
+        <x:v>faulty/nemotron/101.json</x:v>
       </x:c>
       <x:c r="I12" s="11" t="str">
-        <x:v>glm/101.json</x:v>
+        <x:v>faulty/glm/101.json</x:v>
       </x:c>
       <x:c r="J12" s="10" t="n">
         <x:f>COUNTA(G12:I12)</x:f>
@@ -868,13 +868,13 @@
         <x:v>../references/sps_references_export.ris#record-34</x:v>
       </x:c>
       <x:c r="G14" s="11" t="str">
-        <x:v>deepseek/106.json</x:v>
+        <x:v>faulty/deepseek/106.json</x:v>
       </x:c>
       <x:c r="H14" s="11" t="str">
-        <x:v>nemotron/106.json</x:v>
+        <x:v>faulty/nemotron/106.json</x:v>
       </x:c>
       <x:c r="I14" s="11" t="str">
-        <x:v>glm/106.json</x:v>
+        <x:v>faulty/glm/106.json</x:v>
       </x:c>
       <x:c r="J14" s="10" t="n">
         <x:f>COUNTA(G14:I14)</x:f>
@@ -991,13 +991,13 @@
         <x:v>../references/sps_references_export.ris#record-37</x:v>
       </x:c>
       <x:c r="G17" s="11" t="str">
-        <x:v>deepseek/112.json</x:v>
+        <x:v>faulty/deepseek/112.json</x:v>
       </x:c>
       <x:c r="H17" s="11" t="str">
-        <x:v>nemotron/112.json</x:v>
+        <x:v>faulty/nemotron/112.json</x:v>
       </x:c>
       <x:c r="I17" s="11" t="str">
-        <x:v>glm/112.json</x:v>
+        <x:v>faulty/glm/112.json</x:v>
       </x:c>
       <x:c r="J17" s="10" t="n">
         <x:f>COUNTA(G17:I17)</x:f>
@@ -1155,13 +1155,13 @@
         <x:v>../references/sps_references_export.ris#record-43</x:v>
       </x:c>
       <x:c r="G21" s="11" t="str">
-        <x:v>deepseek/121.json</x:v>
+        <x:v>faulty/deepseek/121.json</x:v>
       </x:c>
       <x:c r="H21" s="11" t="str">
-        <x:v>nemotron/121.json</x:v>
+        <x:v>faulty/nemotron/121.json</x:v>
       </x:c>
       <x:c r="I21" s="11" t="str">
-        <x:v>glm/121.json</x:v>
+        <x:v>faulty/glm/121.json</x:v>
       </x:c>
       <x:c r="J21" s="10" t="n">
         <x:f>COUNTA(G21:I21)</x:f>
@@ -1647,13 +1647,13 @@
         <x:v>../references/sps_references_export.ris#record-62</x:v>
       </x:c>
       <x:c r="G33" s="11" t="str">
-        <x:v>deepseek/182.json</x:v>
+        <x:v>faulty/deepseek/182.json</x:v>
       </x:c>
       <x:c r="H33" s="11" t="str">
-        <x:v>nemotron/182.json</x:v>
+        <x:v>faulty/nemotron/182.json</x:v>
       </x:c>
       <x:c r="I33" s="11" t="str">
-        <x:v>glm/182.json</x:v>
+        <x:v>faulty/glm/182.json</x:v>
       </x:c>
       <x:c r="J33" s="10" t="n">
         <x:f>COUNTA(G33:I33)</x:f>
@@ -1811,13 +1811,13 @@
         <x:v>../references/sps_references_export.ris#record-67</x:v>
       </x:c>
       <x:c r="G37" s="11" t="str">
-        <x:v>deepseek/190.json</x:v>
+        <x:v>faulty/deepseek/190.json</x:v>
       </x:c>
       <x:c r="H37" s="11" t="str">
-        <x:v>nemotron/190.json</x:v>
+        <x:v>faulty/nemotron/190.json</x:v>
       </x:c>
       <x:c r="I37" s="11" t="str">
-        <x:v>glm/190.json</x:v>
+        <x:v>faulty/glm/190.json</x:v>
       </x:c>
       <x:c r="J37" s="10" t="n">
         <x:f>COUNTA(G37:I37)</x:f>
@@ -2139,13 +2139,13 @@
         <x:v>../references/sps_references_export.ris#record-79</x:v>
       </x:c>
       <x:c r="G45" s="11" t="str">
-        <x:v>deepseek/223.json</x:v>
+        <x:v>faulty/deepseek/223.json</x:v>
       </x:c>
       <x:c r="H45" s="11" t="str">
-        <x:v>nemotron/223.json</x:v>
+        <x:v>faulty/nemotron/223.json</x:v>
       </x:c>
       <x:c r="I45" s="11" t="str">
-        <x:v>glm/223.json</x:v>
+        <x:v>faulty/glm/223.json</x:v>
       </x:c>
       <x:c r="J45" s="10" t="n">
         <x:f>COUNTA(G45:I45)</x:f>
@@ -2797,13 +2797,13 @@
         <x:v>../references/sps_references_export.ris#record-107</x:v>
       </x:c>
       <x:c r="G61" s="11" t="str">
-        <x:v>deepseek/286.json</x:v>
+        <x:v>faulty/deepseek/286.json</x:v>
       </x:c>
       <x:c r="H61" s="11" t="str">
-        <x:v>nemotron/286.json</x:v>
+        <x:v>faulty/nemotron/286.json</x:v>
       </x:c>
       <x:c r="I61" s="11" t="str">
-        <x:v>glm/286.json</x:v>
+        <x:v>faulty/glm/286.json</x:v>
       </x:c>
       <x:c r="J61" s="10" t="n">
         <x:f>COUNTA(G61:I61)</x:f>
@@ -3084,13 +3084,13 @@
         <x:v>../references/sps_references_export.ris#record-120</x:v>
       </x:c>
       <x:c r="G68" s="11" t="str">
-        <x:v>deepseek/395.json</x:v>
+        <x:v>faulty/deepseek/395.json</x:v>
       </x:c>
       <x:c r="H68" s="11" t="str">
-        <x:v>nemotron/395.json</x:v>
+        <x:v>faulty/nemotron/395.json</x:v>
       </x:c>
       <x:c r="I68" s="11" t="str">
-        <x:v>glm/395.json</x:v>
+        <x:v>faulty/glm/395.json</x:v>
       </x:c>
       <x:c r="J68" s="10" t="n">
         <x:f>COUNTA(G68:I68)</x:f>
@@ -3576,13 +3576,13 @@
         <x:v>../references/sps_references_export.ris#record-134</x:v>
       </x:c>
       <x:c r="G80" s="11" t="str">
-        <x:v>deepseek/429.json</x:v>
+        <x:v>faulty/deepseek/429.json</x:v>
       </x:c>
       <x:c r="H80" s="11" t="str">
-        <x:v>nemotron/429.json</x:v>
+        <x:v>faulty/nemotron/429.json</x:v>
       </x:c>
       <x:c r="I80" s="11" t="str">
-        <x:v>glm/429.json</x:v>
+        <x:v>faulty/glm/429.json</x:v>
       </x:c>
       <x:c r="J80" s="10" t="n">
         <x:f>COUNTA(G80:I80)</x:f>
@@ -4199,13 +4199,13 @@
         <x:v>../references/sps_references_export.ris#record-159</x:v>
       </x:c>
       <x:c r="G95" s="11" t="str">
-        <x:v>deepseek/497.json</x:v>
+        <x:v>faulty/deepseek/497.json</x:v>
       </x:c>
       <x:c r="H95" s="11" t="str">
-        <x:v>nemotron/497.json</x:v>
+        <x:v>faulty/nemotron/497.json</x:v>
       </x:c>
       <x:c r="I95" s="11" t="str">
-        <x:v>glm/497.json</x:v>
+        <x:v>faulty/glm/497.json</x:v>
       </x:c>
       <x:c r="J95" s="10" t="n">
         <x:f>COUNTA(G95:I95)</x:f>
@@ -4584,13 +4584,13 @@
         <x:v>../references/sps_references_export.ris#record-170</x:v>
       </x:c>
       <x:c r="G104" s="11" t="str">
-        <x:v>deepseek/522.json</x:v>
+        <x:v>faulty/deepseek/522.json</x:v>
       </x:c>
       <x:c r="H104" s="11" t="str">
-        <x:v>nemotron/522.json</x:v>
+        <x:v>faulty/nemotron/522.json</x:v>
       </x:c>
       <x:c r="I104" s="11" t="str">
-        <x:v>glm/522.json</x:v>
+        <x:v>faulty/glm/522.json</x:v>
       </x:c>
       <x:c r="J104" s="10" t="n">
         <x:f>COUNTA(G104:I104)</x:f>
@@ -4627,13 +4627,13 @@
         <x:v>../references/sps_references_export.ris#record-171</x:v>
       </x:c>
       <x:c r="G105" s="11" t="str">
-        <x:v>deepseek/524.json</x:v>
+        <x:v>faulty/deepseek/524.json</x:v>
       </x:c>
       <x:c r="H105" s="11" t="str">
-        <x:v>nemotron/524.json</x:v>
+        <x:v>faulty/nemotron/524.json</x:v>
       </x:c>
       <x:c r="I105" s="11" t="str">
-        <x:v>glm/524.json</x:v>
+        <x:v>faulty/glm/524.json</x:v>
       </x:c>
       <x:c r="J105" s="10" t="n">
         <x:f>COUNTA(G105:I105)</x:f>
@@ -5010,13 +5010,13 @@
         <x:v>../references/sps_references_export.ris#record-185</x:v>
       </x:c>
       <x:c r="G114" s="11" t="str">
-        <x:v>deepseek/551.json</x:v>
+        <x:v>faulty/deepseek/551.json</x:v>
       </x:c>
       <x:c r="H114" s="11" t="str">
-        <x:v>nemotron/551.json</x:v>
+        <x:v>faulty/nemotron/551.json</x:v>
       </x:c>
       <x:c r="I114" s="11" t="str">
-        <x:v>glm/551.json</x:v>
+        <x:v>faulty/glm/551.json</x:v>
       </x:c>
       <x:c r="J114" s="10" t="n">
         <x:f>COUNTA(G114:I114)</x:f>
@@ -5907,13 +5907,13 @@
         <x:v>../references/sps_references_export.ris#record-214</x:v>
       </x:c>
       <x:c r="G135" s="11" t="str">
-        <x:v>deepseek/608.json</x:v>
+        <x:v>faulty/deepseek/608.json</x:v>
       </x:c>
       <x:c r="H135" s="11" t="str">
-        <x:v>nemotron/608.json</x:v>
+        <x:v>faulty/nemotron/608.json</x:v>
       </x:c>
       <x:c r="I135" s="11" t="str">
-        <x:v>glm/608.json</x:v>
+        <x:v>faulty/glm/608.json</x:v>
       </x:c>
       <x:c r="J135" s="10" t="n">
         <x:f>COUNTA(G135:I135)</x:f>
@@ -6071,13 +6071,13 @@
         <x:v>../references/sps_references_export.ris#record-220</x:v>
       </x:c>
       <x:c r="G139" s="11" t="str">
-        <x:v>deepseek/621.json</x:v>
+        <x:v>faulty/deepseek/621.json</x:v>
       </x:c>
       <x:c r="H139" s="11" t="str">
-        <x:v>nemotron/621.json</x:v>
+        <x:v>faulty/nemotron/621.json</x:v>
       </x:c>
       <x:c r="I139" s="11" t="str">
-        <x:v>glm/621.json</x:v>
+        <x:v>faulty/glm/621.json</x:v>
       </x:c>
       <x:c r="J139" s="10" t="n">
         <x:f>COUNTA(G139:I139)</x:f>
@@ -6112,13 +6112,13 @@
         <x:v>../references/sps_references_export.ris#record-221</x:v>
       </x:c>
       <x:c r="G140" s="11" t="str">
-        <x:v>deepseek/623.json</x:v>
+        <x:v>faulty/deepseek/623.json</x:v>
       </x:c>
       <x:c r="H140" s="11" t="str">
-        <x:v>nemotron/623.json</x:v>
+        <x:v>faulty/nemotron/623.json</x:v>
       </x:c>
       <x:c r="I140" s="11" t="str">
-        <x:v>glm/623.json</x:v>
+        <x:v>faulty/glm/623.json</x:v>
       </x:c>
       <x:c r="J140" s="10" t="n">
         <x:f>COUNTA(G140:I140)</x:f>
@@ -6651,13 +6651,13 @@
         <x:v>../references/sps_references_export.ris#record-239</x:v>
       </x:c>
       <x:c r="G153" s="11" t="str">
-        <x:v>deepseek/658.json</x:v>
+        <x:v>faulty/deepseek/658.json</x:v>
       </x:c>
       <x:c r="H153" s="11" t="str">
-        <x:v>nemotron/658.json</x:v>
+        <x:v>faulty/nemotron/658.json</x:v>
       </x:c>
       <x:c r="I153" s="11" t="str">
-        <x:v>glm/658.json</x:v>
+        <x:v>faulty/glm/658.json</x:v>
       </x:c>
       <x:c r="J153" s="10" t="n">
         <x:f>COUNTA(G153:I153)</x:f>
@@ -6909,13 +6909,13 @@
         <x:v>../references/sps_references_export.ris#record-251</x:v>
       </x:c>
       <x:c r="G159" s="11" t="str">
-        <x:v>deepseek/680.json</x:v>
+        <x:v>faulty/deepseek/680.json</x:v>
       </x:c>
       <x:c r="H159" s="11" t="str">
-        <x:v>nemotron/680.json</x:v>
+        <x:v>faulty/nemotron/680.json</x:v>
       </x:c>
       <x:c r="I159" s="11" t="str">
-        <x:v>glm/680.json</x:v>
+        <x:v>faulty/glm/680.json</x:v>
       </x:c>
       <x:c r="J159" s="10" t="n">
         <x:f>COUNTA(G159:I159)</x:f>
@@ -6952,13 +6952,13 @@
         <x:v>../references/sps_references_export.ris#record-252</x:v>
       </x:c>
       <x:c r="G160" s="11" t="str">
-        <x:v>deepseek/682.json</x:v>
+        <x:v>faulty/deepseek/682.json</x:v>
       </x:c>
       <x:c r="H160" s="11" t="str">
-        <x:v>nemotron/682.json</x:v>
+        <x:v>faulty/nemotron/682.json</x:v>
       </x:c>
       <x:c r="I160" s="11" t="str">
-        <x:v>glm/682.json</x:v>
+        <x:v>faulty/glm/682.json</x:v>
       </x:c>
       <x:c r="J160" s="10" t="n">
         <x:f>COUNTA(G160:I160)</x:f>
@@ -7122,13 +7122,13 @@
         <x:v>../references/sps_references_export.ris#record-259</x:v>
       </x:c>
       <x:c r="G164" s="11" t="str">
-        <x:v>deepseek/705.json</x:v>
+        <x:v>faulty/deepseek/705.json</x:v>
       </x:c>
       <x:c r="H164" s="11" t="str">
-        <x:v>nemotron/705.json</x:v>
+        <x:v>faulty/nemotron/705.json</x:v>
       </x:c>
       <x:c r="I164" s="11" t="str">
-        <x:v>glm/705.json</x:v>
+        <x:v>faulty/glm/705.json</x:v>
       </x:c>
       <x:c r="J164" s="10" t="n">
         <x:f>COUNTA(G164:I164)</x:f>
@@ -7421,13 +7421,13 @@
         <x:v>../references/sps_references_export.ris#record-271</x:v>
       </x:c>
       <x:c r="G171" s="11" t="str">
-        <x:v>deepseek/736.json</x:v>
+        <x:v>faulty/deepseek/736.json</x:v>
       </x:c>
       <x:c r="H171" s="11" t="str">
-        <x:v>nemotron/736.json</x:v>
+        <x:v>faulty/nemotron/736.json</x:v>
       </x:c>
       <x:c r="I171" s="11" t="str">
-        <x:v>glm/736.json</x:v>
+        <x:v>faulty/glm/736.json</x:v>
       </x:c>
       <x:c r="J171" s="10" t="n">
         <x:f>COUNTA(G171:I171)</x:f>
@@ -7464,13 +7464,13 @@
         <x:v>../references/sps_references_export.ris#record-277</x:v>
       </x:c>
       <x:c r="G172" s="11" t="str">
-        <x:v>deepseek/754.json</x:v>
+        <x:v>faulty/deepseek/754.json</x:v>
       </x:c>
       <x:c r="H172" s="11" t="str">
-        <x:v>nemotron/754.json</x:v>
+        <x:v>faulty/nemotron/754.json</x:v>
       </x:c>
       <x:c r="I172" s="11" t="str">
-        <x:v>glm/754.json</x:v>
+        <x:v>faulty/glm/754.json</x:v>
       </x:c>
       <x:c r="J172" s="10" t="n">
         <x:f>COUNTA(G172:I172)</x:f>
@@ -7978,13 +7978,13 @@
         <x:v>../references/sps_references_export.ris#record-297</x:v>
       </x:c>
       <x:c r="G184" s="11" t="str">
-        <x:v>deepseek/815.json</x:v>
+        <x:v>faulty/deepseek/815.json</x:v>
       </x:c>
       <x:c r="H184" s="11" t="str">
-        <x:v>nemotron/815.json</x:v>
+        <x:v>faulty/nemotron/815.json</x:v>
       </x:c>
       <x:c r="I184" s="11" t="str">
-        <x:v>glm/815.json</x:v>
+        <x:v>faulty/glm/815.json</x:v>
       </x:c>
       <x:c r="J184" s="10" t="n">
         <x:f>COUNTA(G184:I184)</x:f>
@@ -8021,13 +8021,13 @@
         <x:v>../references/sps_references_export.ris#record-300</x:v>
       </x:c>
       <x:c r="G185" s="11" t="str">
-        <x:v>deepseek/822.json</x:v>
+        <x:v>faulty/deepseek/822.json</x:v>
       </x:c>
       <x:c r="H185" s="11" t="str">
-        <x:v>nemotron/822.json</x:v>
+        <x:v>faulty/nemotron/822.json</x:v>
       </x:c>
       <x:c r="I185" s="11" t="str">
-        <x:v>glm/822.json</x:v>
+        <x:v>faulty/glm/822.json</x:v>
       </x:c>
       <x:c r="J185" s="10" t="n">
         <x:f>COUNTA(G185:I185)</x:f>
@@ -8193,13 +8193,13 @@
         <x:v>../references/sps_references_export.ris#record-306</x:v>
       </x:c>
       <x:c r="G189" s="11" t="str">
-        <x:v>deepseek/830.json</x:v>
+        <x:v>faulty/deepseek/830.json</x:v>
       </x:c>
       <x:c r="H189" s="11" t="str">
-        <x:v>nemotron/830.json</x:v>
+        <x:v>faulty/nemotron/830.json</x:v>
       </x:c>
       <x:c r="I189" s="11" t="str">
-        <x:v>glm/830.json</x:v>
+        <x:v>faulty/glm/830.json</x:v>
       </x:c>
       <x:c r="J189" s="10" t="n">
         <x:f>COUNTA(G189:I189)</x:f>
@@ -8277,13 +8277,13 @@
         <x:v>../references/sps_references_export.ris#record-309</x:v>
       </x:c>
       <x:c r="G191" s="11" t="str">
-        <x:v>deepseek/834.json</x:v>
+        <x:v>faulty/deepseek/834.json</x:v>
       </x:c>
       <x:c r="H191" s="11" t="str">
-        <x:v>nemotron/834.json</x:v>
+        <x:v>faulty/nemotron/834.json</x:v>
       </x:c>
       <x:c r="I191" s="11" t="str">
-        <x:v>glm/834.json</x:v>
+        <x:v>faulty/glm/834.json</x:v>
       </x:c>
       <x:c r="J191" s="10" t="n">
         <x:f>COUNTA(G191:I191)</x:f>
@@ -8363,13 +8363,13 @@
         <x:v>../references/sps_references_export.ris#record-311</x:v>
       </x:c>
       <x:c r="G193" s="11" t="str">
-        <x:v>deepseek/837.json</x:v>
+        <x:v>faulty/deepseek/837.json</x:v>
       </x:c>
       <x:c r="H193" s="11" t="str">
-        <x:v>nemotron/837.json</x:v>
+        <x:v>faulty/nemotron/837.json</x:v>
       </x:c>
       <x:c r="I193" s="11" t="str">
-        <x:v>glm/837.json</x:v>
+        <x:v>faulty/glm/837.json</x:v>
       </x:c>
       <x:c r="J193" s="10" t="n">
         <x:f>COUNTA(G193:I193)</x:f>
@@ -8576,13 +8576,13 @@
         <x:v>../references/sps_references_export.ris#record-318</x:v>
       </x:c>
       <x:c r="G198" s="11" t="str">
-        <x:v>deepseek/857.json</x:v>
+        <x:v>faulty/deepseek/857.json</x:v>
       </x:c>
       <x:c r="H198" s="11" t="str">
-        <x:v>nemotron/857.json</x:v>
+        <x:v>faulty/nemotron/857.json</x:v>
       </x:c>
       <x:c r="I198" s="11" t="str">
-        <x:v>glm/857.json</x:v>
+        <x:v>faulty/glm/857.json</x:v>
       </x:c>
       <x:c r="J198" s="10" t="n">
         <x:f>COUNTA(G198:I198)</x:f>
@@ -8703,13 +8703,13 @@
         <x:v>../references/sps_references_export.ris#record-321</x:v>
       </x:c>
       <x:c r="G201" s="11" t="str">
-        <x:v>deepseek/862.json</x:v>
+        <x:v>faulty/deepseek/862.json</x:v>
       </x:c>
       <x:c r="H201" s="11" t="str">
-        <x:v>nemotron/862.json</x:v>
+        <x:v>faulty/nemotron/862.json</x:v>
       </x:c>
       <x:c r="I201" s="11" t="str">
-        <x:v>glm/862.json</x:v>
+        <x:v>faulty/glm/862.json</x:v>
       </x:c>
       <x:c r="J201" s="10" t="n">
         <x:f>COUNTA(G201:I201)</x:f>
@@ -8746,13 +8746,13 @@
         <x:v>../references/sps_references_export.ris#record-322</x:v>
       </x:c>
       <x:c r="G202" s="11" t="str">
-        <x:v>deepseek/867.json</x:v>
+        <x:v>faulty/deepseek/867.json</x:v>
       </x:c>
       <x:c r="H202" s="11" t="str">
-        <x:v>nemotron/867.json</x:v>
+        <x:v>faulty/nemotron/867.json</x:v>
       </x:c>
       <x:c r="I202" s="11" t="str">
-        <x:v>glm/867.json</x:v>
+        <x:v>faulty/glm/867.json</x:v>
       </x:c>
       <x:c r="J202" s="10" t="n">
         <x:f>COUNTA(G202:I202)</x:f>
@@ -8959,13 +8959,13 @@
         <x:v>../references/sps_references_export.ris#record-327</x:v>
       </x:c>
       <x:c r="G207" s="11" t="str">
-        <x:v>deepseek/875.json</x:v>
+        <x:v>faulty/deepseek/875.json</x:v>
       </x:c>
       <x:c r="H207" s="11" t="str">
-        <x:v>nemotron/875.json</x:v>
+        <x:v>faulty/nemotron/875.json</x:v>
       </x:c>
       <x:c r="I207" s="11" t="str">
-        <x:v>glm/875.json</x:v>
+        <x:v>faulty/glm/875.json</x:v>
       </x:c>
       <x:c r="J207" s="10" t="n">
         <x:f>COUNTA(G207:I207)</x:f>
@@ -9430,13 +9430,13 @@
         <x:v>../references/sps_references_export.ris#record-340</x:v>
       </x:c>
       <x:c r="G218" s="11" t="str">
-        <x:v>deepseek/897.json</x:v>
+        <x:v>faulty/deepseek/897.json</x:v>
       </x:c>
       <x:c r="H218" s="11" t="str">
-        <x:v>nemotron/897.json</x:v>
+        <x:v>faulty/nemotron/897.json</x:v>
       </x:c>
       <x:c r="I218" s="11" t="str">
-        <x:v>glm/897.json</x:v>
+        <x:v>faulty/glm/897.json</x:v>
       </x:c>
       <x:c r="J218" s="10" t="n">
         <x:f>COUNTA(G218:I218)</x:f>
@@ -10112,13 +10112,13 @@
         <x:v>../references/sps_references_export.ris#record-366</x:v>
       </x:c>
       <x:c r="G234" s="11" t="str">
-        <x:v>deepseek/960.json</x:v>
+        <x:v>faulty/deepseek/960.json</x:v>
       </x:c>
       <x:c r="H234" s="11" t="str">
-        <x:v>nemotron/960.json</x:v>
+        <x:v>faulty/nemotron/960.json</x:v>
       </x:c>
       <x:c r="I234" s="11" t="str">
-        <x:v>glm/960.json</x:v>
+        <x:v>faulty/glm/960.json</x:v>
       </x:c>
       <x:c r="J234" s="10" t="n">
         <x:f>COUNTA(G234:I234)</x:f>
@@ -10958,13 +10958,13 @@
         <x:v>../references/sps_references_export.ris#record-425</x:v>
       </x:c>
       <x:c r="G254" s="11" t="str">
-        <x:v>deepseek/1248.json</x:v>
+        <x:v>faulty/deepseek/1248.json</x:v>
       </x:c>
       <x:c r="H254" s="11" t="str">
-        <x:v>nemotron/1248.json</x:v>
+        <x:v>faulty/nemotron/1248.json</x:v>
       </x:c>
       <x:c r="I254" s="11" t="str">
-        <x:v>glm/1248.json</x:v>
+        <x:v>faulty/glm/1248.json</x:v>
       </x:c>
       <x:c r="J254" s="10" t="n">
         <x:f>COUNTA(G254:I254)</x:f>
@@ -11171,13 +11171,13 @@
         <x:v>../references/sps_references_export.ris#record-433</x:v>
       </x:c>
       <x:c r="G259" s="11" t="str">
-        <x:v>deepseek/1298.json</x:v>
+        <x:v>faulty/deepseek/1298.json</x:v>
       </x:c>
       <x:c r="H259" s="11" t="str">
-        <x:v>nemotron/1298.json</x:v>
+        <x:v>faulty/nemotron/1298.json</x:v>
       </x:c>
       <x:c r="I259" s="11" t="str">
-        <x:v>glm/1298.json</x:v>
+        <x:v>faulty/glm/1298.json</x:v>
       </x:c>
       <x:c r="J259" s="10" t="n">
         <x:f>COUNTA(G259:I259)</x:f>
@@ -11214,13 +11214,13 @@
         <x:v>../references/sps_references_export.ris#record-435</x:v>
       </x:c>
       <x:c r="G260" s="11" t="str">
-        <x:v>deepseek/1326.json</x:v>
+        <x:v>faulty/deepseek/1326.json</x:v>
       </x:c>
       <x:c r="H260" s="11" t="str">
-        <x:v>nemotron/1326.json</x:v>
+        <x:v>faulty/nemotron/1326.json</x:v>
       </x:c>
       <x:c r="I260" s="11" t="str">
-        <x:v>glm/1326.json</x:v>
+        <x:v>faulty/glm/1326.json</x:v>
       </x:c>
       <x:c r="J260" s="10" t="n">
         <x:f>COUNTA(G260:I260)</x:f>
@@ -11382,13 +11382,13 @@
         <x:v>../references/sps_references_export.ris#record-446</x:v>
       </x:c>
       <x:c r="G264" s="11" t="str">
-        <x:v>deepseek/1372.json</x:v>
+        <x:v>faulty/deepseek/1372.json</x:v>
       </x:c>
       <x:c r="H264" s="11" t="str">
-        <x:v>nemotron/1372.json</x:v>
+        <x:v>faulty/nemotron/1372.json</x:v>
       </x:c>
       <x:c r="I264" s="11" t="str">
-        <x:v>glm/1372.json</x:v>
+        <x:v>faulty/glm/1372.json</x:v>
       </x:c>
       <x:c r="J264" s="10" t="n">
         <x:f>COUNTA(G264:I264)</x:f>
@@ -11423,13 +11423,13 @@
         <x:v>../references/sps_references_export.ris#record-453</x:v>
       </x:c>
       <x:c r="G265" s="11" t="str">
-        <x:v>deepseek/1394.json</x:v>
+        <x:v>faulty/deepseek/1394.json</x:v>
       </x:c>
       <x:c r="H265" s="11" t="str">
-        <x:v>nemotron/1394.json</x:v>
+        <x:v>faulty/nemotron/1394.json</x:v>
       </x:c>
       <x:c r="I265" s="11" t="str">
-        <x:v>glm/1394.json</x:v>
+        <x:v>faulty/glm/1394.json</x:v>
       </x:c>
       <x:c r="J265" s="10" t="n">
         <x:f>COUNTA(G265:I265)</x:f>
@@ -11466,13 +11466,13 @@
         <x:v>../references/sps_references_export.ris#record-458</x:v>
       </x:c>
       <x:c r="G266" s="11" t="str">
-        <x:v>deepseek/1401.json</x:v>
+        <x:v>faulty/deepseek/1401.json</x:v>
       </x:c>
       <x:c r="H266" s="11" t="str">
-        <x:v>nemotron/1401.json</x:v>
+        <x:v>faulty/nemotron/1401.json</x:v>
       </x:c>
       <x:c r="I266" s="11" t="str">
-        <x:v>glm/1401.json</x:v>
+        <x:v>faulty/glm/1401.json</x:v>
       </x:c>
       <x:c r="J266" s="10" t="n">
         <x:f>COUNTA(G266:I266)</x:f>
@@ -11677,13 +11677,13 @@
         <x:v>../references/sps_references_export.ris#record-492</x:v>
       </x:c>
       <x:c r="G271" s="11" t="str">
-        <x:v>deepseek/1610.json</x:v>
+        <x:v>faulty/deepseek/1610.json</x:v>
       </x:c>
       <x:c r="H271" s="11" t="str">
-        <x:v>nemotron/1610.json</x:v>
+        <x:v>faulty/nemotron/1610.json</x:v>
       </x:c>
       <x:c r="I271" s="11" t="str">
-        <x:v>glm/1610.json</x:v>
+        <x:v>faulty/glm/1610.json</x:v>
       </x:c>
       <x:c r="J271" s="10" t="n">
         <x:f>COUNTA(G271:I271)</x:f>
@@ -12347,13 +12347,13 @@
         <x:v>../references/sps_references_export.ris#record-521</x:v>
       </x:c>
       <x:c r="G287" s="11" t="str">
-        <x:v>deepseek/1739.json</x:v>
+        <x:v>faulty/deepseek/1739.json</x:v>
       </x:c>
       <x:c r="H287" s="11" t="str">
-        <x:v>nemotron/1739.json</x:v>
+        <x:v>faulty/nemotron/1739.json</x:v>
       </x:c>
       <x:c r="I287" s="11" t="str">
-        <x:v>glm/1739.json</x:v>
+        <x:v>faulty/glm/1739.json</x:v>
       </x:c>
       <x:c r="J287" s="10" t="n">
         <x:f>COUNTA(G287:I287)</x:f>
@@ -12433,13 +12433,13 @@
         <x:v>../references/sps_references_export.ris#record-523</x:v>
       </x:c>
       <x:c r="G289" s="11" t="str">
-        <x:v>deepseek/1742.json</x:v>
+        <x:v>faulty/deepseek/1742.json</x:v>
       </x:c>
       <x:c r="H289" s="11" t="str">
-        <x:v>nemotron/1742.json</x:v>
+        <x:v>faulty/nemotron/1742.json</x:v>
       </x:c>
       <x:c r="I289" s="11" t="str">
-        <x:v>glm/1742.json</x:v>
+        <x:v>faulty/glm/1742.json</x:v>
       </x:c>
       <x:c r="J289" s="10" t="n">
         <x:f>COUNTA(G289:I289)</x:f>
@@ -12902,13 +12902,13 @@
         <x:v>../references/sps_references_export.ris#record-548</x:v>
       </x:c>
       <x:c r="G300" s="11" t="str">
-        <x:v>deepseek/1841.json</x:v>
+        <x:v>faulty/deepseek/1841.json</x:v>
       </x:c>
       <x:c r="H300" s="11" t="str">
-        <x:v>nemotron/1841.json</x:v>
+        <x:v>faulty/nemotron/1841.json</x:v>
       </x:c>
       <x:c r="I300" s="11" t="str">
-        <x:v>glm/1841.json</x:v>
+        <x:v>faulty/glm/1841.json</x:v>
       </x:c>
       <x:c r="J300" s="10" t="n">
         <x:f>COUNTA(G300:I300)</x:f>
@@ -13582,13 +13582,13 @@
         <x:v>../references/sps_references_export.ris#record-589</x:v>
       </x:c>
       <x:c r="G316" s="11" t="str">
-        <x:v>deepseek/1962.json</x:v>
+        <x:v>faulty/deepseek/1962.json</x:v>
       </x:c>
       <x:c r="H316" s="11" t="str">
-        <x:v>nemotron/1962.json</x:v>
+        <x:v>faulty/nemotron/1962.json</x:v>
       </x:c>
       <x:c r="I316" s="11" t="str">
-        <x:v>glm/1962.json</x:v>
+        <x:v>faulty/glm/1962.json</x:v>
       </x:c>
       <x:c r="J316" s="10" t="n">
         <x:f>COUNTA(G316:I316)</x:f>
@@ -14174,13 +14174,13 @@
         <x:v>../references/sps_references_export.ris#record-604</x:v>
       </x:c>
       <x:c r="G330" s="11" t="str">
-        <x:v>deepseek/2461.json</x:v>
+        <x:v>faulty/deepseek/2461.json</x:v>
       </x:c>
       <x:c r="H330" s="11" t="str">
-        <x:v>nemotron/2461.json</x:v>
+        <x:v>faulty/nemotron/2461.json</x:v>
       </x:c>
       <x:c r="I330" s="11" t="str">
-        <x:v>glm/2461.json</x:v>
+        <x:v>faulty/glm/2461.json</x:v>
       </x:c>
       <x:c r="J330" s="10" t="n">
         <x:f>COUNTA(G330:I330)</x:f>
@@ -14346,13 +14346,13 @@
         <x:v>../references/sps_references_export.ris#record-611</x:v>
       </x:c>
       <x:c r="G334" s="11" t="str">
-        <x:v>deepseek/2592.json</x:v>
+        <x:v>faulty/deepseek/2592.json</x:v>
       </x:c>
       <x:c r="H334" s="11" t="str">
-        <x:v>nemotron/2592.json</x:v>
+        <x:v>faulty/nemotron/2592.json</x:v>
       </x:c>
       <x:c r="I334" s="11" t="str">
-        <x:v>glm/2592.json</x:v>
+        <x:v>faulty/glm/2592.json</x:v>
       </x:c>
       <x:c r="J334" s="10" t="n">
         <x:f>COUNTA(G334:I334)</x:f>
@@ -14432,13 +14432,13 @@
         <x:v>../references/sps_references_export.ris#record-614</x:v>
       </x:c>
       <x:c r="G336" s="11" t="str">
-        <x:v>deepseek/2610.json</x:v>
+        <x:v>faulty/deepseek/2610.json</x:v>
       </x:c>
       <x:c r="H336" s="11" t="str">
-        <x:v>nemotron/2610.json</x:v>
+        <x:v>faulty/nemotron/2610.json</x:v>
       </x:c>
       <x:c r="I336" s="11" t="str">
-        <x:v>glm/2610.json</x:v>
+        <x:v>faulty/glm/2610.json</x:v>
       </x:c>
       <x:c r="J336" s="10" t="n">
         <x:f>COUNTA(G336:I336)</x:f>
@@ -14475,13 +14475,13 @@
         <x:v>../references/sps_references_export.ris#record-615</x:v>
       </x:c>
       <x:c r="G337" s="11" t="str">
-        <x:v>deepseek/2615.json</x:v>
+        <x:v>faulty/deepseek/2615.json</x:v>
       </x:c>
       <x:c r="H337" s="11" t="str">
-        <x:v>nemotron/2615.json</x:v>
+        <x:v>faulty/nemotron/2615.json</x:v>
       </x:c>
       <x:c r="I337" s="11" t="str">
-        <x:v>glm/2615.json</x:v>
+        <x:v>faulty/glm/2615.json</x:v>
       </x:c>
       <x:c r="J337" s="10" t="n">
         <x:f>COUNTA(G337:I337)</x:f>
@@ -14647,13 +14647,13 @@
         <x:v>../references/sps_references_export.ris#record-621</x:v>
       </x:c>
       <x:c r="G341" s="11" t="str">
-        <x:v>deepseek/2658.json</x:v>
+        <x:v>faulty/deepseek/2658.json</x:v>
       </x:c>
       <x:c r="H341" s="11" t="str">
-        <x:v>nemotron/2658.json</x:v>
+        <x:v>faulty/nemotron/2658.json</x:v>
       </x:c>
       <x:c r="I341" s="11" t="str">
-        <x:v>glm/2658.json</x:v>
+        <x:v>faulty/glm/2658.json</x:v>
       </x:c>
       <x:c r="J341" s="10" t="n">
         <x:f>COUNTA(G341:I341)</x:f>
@@ -15075,13 +15075,13 @@
         <x:v>../references/sps_references_export.ris#record-632</x:v>
       </x:c>
       <x:c r="G351" s="11" t="str">
-        <x:v>deepseek/2879.json</x:v>
+        <x:v>faulty/deepseek/2879.json</x:v>
       </x:c>
       <x:c r="H351" s="11" t="str">
-        <x:v>nemotron/2879.json</x:v>
+        <x:v>faulty/nemotron/2879.json</x:v>
       </x:c>
       <x:c r="I351" s="11" t="str">
-        <x:v>glm/2879.json</x:v>
+        <x:v>faulty/glm/2879.json</x:v>
       </x:c>
       <x:c r="J351" s="10" t="n">
         <x:f>COUNTA(G351:I351)</x:f>
@@ -15118,13 +15118,13 @@
         <x:v>../references/sps_references_export.ris#record-633</x:v>
       </x:c>
       <x:c r="G352" s="11" t="str">
-        <x:v>deepseek/2885.json</x:v>
+        <x:v>faulty/deepseek/2885.json</x:v>
       </x:c>
       <x:c r="H352" s="11" t="str">
-        <x:v>nemotron/2885.json</x:v>
+        <x:v>faulty/nemotron/2885.json</x:v>
       </x:c>
       <x:c r="I352" s="11" t="str">
-        <x:v>glm/2885.json</x:v>
+        <x:v>faulty/glm/2885.json</x:v>
       </x:c>
       <x:c r="J352" s="10" t="n">
         <x:f>COUNTA(G352:I352)</x:f>
@@ -15376,13 +15376,13 @@
         <x:v>../references/sps_references_export.ris#record-644</x:v>
       </x:c>
       <x:c r="G358" s="11" t="str">
-        <x:v>deepseek/3135.json</x:v>
+        <x:v>faulty/deepseek/3135.json</x:v>
       </x:c>
       <x:c r="H358" s="11" t="str">
-        <x:v>nemotron/3135.json</x:v>
+        <x:v>faulty/nemotron/3135.json</x:v>
       </x:c>
       <x:c r="I358" s="11" t="str">
-        <x:v>glm/3135.json</x:v>
+        <x:v>faulty/glm/3135.json</x:v>
       </x:c>
       <x:c r="J358" s="10" t="n">
         <x:f>COUNTA(G358:I358)</x:f>
@@ -15419,13 +15419,13 @@
         <x:v>../references/sps_references_export.ris#record-645</x:v>
       </x:c>
       <x:c r="G359" s="11" t="str">
-        <x:v>deepseek/3136.json</x:v>
+        <x:v>faulty/deepseek/3136.json</x:v>
       </x:c>
       <x:c r="H359" s="11" t="str">
-        <x:v>nemotron/3136.json</x:v>
+        <x:v>faulty/nemotron/3136.json</x:v>
       </x:c>
       <x:c r="I359" s="11" t="str">
-        <x:v>glm/3136.json</x:v>
+        <x:v>faulty/glm/3136.json</x:v>
       </x:c>
       <x:c r="J359" s="10" t="n">
         <x:f>COUNTA(G359:I359)</x:f>
@@ -15710,13 +15710,13 @@
         <x:v>../references/sps_references_export.ris#record-659</x:v>
       </x:c>
       <x:c r="G366" s="11" t="str">
-        <x:v>deepseek/5142.json</x:v>
+        <x:v>faulty/deepseek/5142.json</x:v>
       </x:c>
       <x:c r="H366" s="11" t="str">
-        <x:v>nemotron/5142.json</x:v>
+        <x:v>faulty/nemotron/5142.json</x:v>
       </x:c>
       <x:c r="I366" s="11" t="str">
-        <x:v>glm/5142.json</x:v>
+        <x:v>faulty/glm/5142.json</x:v>
       </x:c>
       <x:c r="J366" s="10" t="n">
         <x:f>COUNTA(G366:I366)</x:f>
@@ -15794,13 +15794,13 @@
         <x:v>../references/sps_references_export.ris#record-663</x:v>
       </x:c>
       <x:c r="G368" s="11" t="str">
-        <x:v>deepseek/5191.json</x:v>
+        <x:v>faulty/deepseek/5191.json</x:v>
       </x:c>
       <x:c r="H368" s="11" t="str">
-        <x:v>nemotron/5191.json</x:v>
+        <x:v>faulty/nemotron/5191.json</x:v>
       </x:c>
       <x:c r="I368" s="11" t="str">
-        <x:v>glm/5191.json</x:v>
+        <x:v>faulty/glm/5191.json</x:v>
       </x:c>
       <x:c r="J368" s="10" t="n">
         <x:f>COUNTA(G368:I368)</x:f>
@@ -15835,13 +15835,13 @@
         <x:v>../references/sps_references_export.ris#record-665</x:v>
       </x:c>
       <x:c r="G369" s="11" t="str">
-        <x:v>deepseek/5219.json</x:v>
+        <x:v>faulty/deepseek/5219.json</x:v>
       </x:c>
       <x:c r="H369" s="11" t="str">
-        <x:v>nemotron/5219.json</x:v>
+        <x:v>faulty/nemotron/5219.json</x:v>
       </x:c>
       <x:c r="I369" s="11" t="str">
-        <x:v>glm/5219.json</x:v>
+        <x:v>faulty/glm/5219.json</x:v>
       </x:c>
       <x:c r="J369" s="10" t="n">
         <x:f>COUNTA(G369:I369)</x:f>
@@ -15878,13 +15878,13 @@
         <x:v>../references/sps_references_export.ris#record-666</x:v>
       </x:c>
       <x:c r="G370" s="11" t="str">
-        <x:v>deepseek/5230.json</x:v>
+        <x:v>faulty/deepseek/5230.json</x:v>
       </x:c>
       <x:c r="H370" s="11" t="str">
-        <x:v>nemotron/5230.json</x:v>
+        <x:v>faulty/nemotron/5230.json</x:v>
       </x:c>
       <x:c r="I370" s="11" t="str">
-        <x:v>glm/5230.json</x:v>
+        <x:v>faulty/glm/5230.json</x:v>
       </x:c>
       <x:c r="J370" s="10" t="n">
         <x:f>COUNTA(G370:I370)</x:f>
@@ -15921,13 +15921,13 @@
         <x:v>../references/sps_references_export.ris#record-669</x:v>
       </x:c>
       <x:c r="G371" s="11" t="str">
-        <x:v>deepseek/5243.json</x:v>
+        <x:v>faulty/deepseek/5243.json</x:v>
       </x:c>
       <x:c r="H371" s="11" t="str">
-        <x:v>nemotron/5243.json</x:v>
+        <x:v>faulty/nemotron/5243.json</x:v>
       </x:c>
       <x:c r="I371" s="11" t="str">
-        <x:v>glm/5243.json</x:v>
+        <x:v>faulty/glm/5243.json</x:v>
       </x:c>
       <x:c r="J371" s="10" t="n">
         <x:f>COUNTA(G371:I371)</x:f>
@@ -15962,13 +15962,13 @@
         <x:v>../references/sps_references_export.ris#record-670</x:v>
       </x:c>
       <x:c r="G372" s="11" t="str">
-        <x:v>deepseek/5254.json</x:v>
+        <x:v>faulty/deepseek/5254.json</x:v>
       </x:c>
       <x:c r="H372" s="11" t="str">
-        <x:v>nemotron/5254.json</x:v>
+        <x:v>faulty/nemotron/5254.json</x:v>
       </x:c>
       <x:c r="I372" s="11" t="str">
-        <x:v>glm/5254.json</x:v>
+        <x:v>faulty/glm/5254.json</x:v>
       </x:c>
       <x:c r="J372" s="10" t="n">
         <x:f>COUNTA(G372:I372)</x:f>
@@ -16046,13 +16046,13 @@
         <x:v>../references/sps_references_export.ris#record-688</x:v>
       </x:c>
       <x:c r="G374" s="11" t="str">
-        <x:v>deepseek/5499.json</x:v>
+        <x:v>faulty/deepseek/5499.json</x:v>
       </x:c>
       <x:c r="H374" s="11" t="str">
-        <x:v>nemotron/5499.json</x:v>
+        <x:v>faulty/nemotron/5499.json</x:v>
       </x:c>
       <x:c r="I374" s="11" t="str">
-        <x:v>glm/5499.json</x:v>
+        <x:v>faulty/glm/5499.json</x:v>
       </x:c>
       <x:c r="J374" s="10" t="n">
         <x:f>COUNTA(G374:I374)</x:f>
@@ -16251,13 +16251,13 @@
         <x:v>../references/sps_references_export.ris#record-718</x:v>
       </x:c>
       <x:c r="G379" s="11" t="str">
-        <x:v>deepseek/5985.json</x:v>
+        <x:v>faulty/deepseek/5985.json</x:v>
       </x:c>
       <x:c r="H379" s="11" t="str">
-        <x:v>nemotron/5985.json</x:v>
+        <x:v>faulty/nemotron/5985.json</x:v>
       </x:c>
       <x:c r="I379" s="11" t="str">
-        <x:v>glm/5985.json</x:v>
+        <x:v>faulty/glm/5985.json</x:v>
       </x:c>
       <x:c r="J379" s="10" t="n">
         <x:f>COUNTA(G379:I379)</x:f>
@@ -16589,13 +16589,13 @@
         <x:v>../references/sps_references_export.ris#record-734</x:v>
       </x:c>
       <x:c r="G387" s="11" t="str">
-        <x:v>deepseek/6152.json</x:v>
+        <x:v>faulty/deepseek/6152.json</x:v>
       </x:c>
       <x:c r="H387" s="11" t="str">
-        <x:v>nemotron/6152.json</x:v>
+        <x:v>faulty/nemotron/6152.json</x:v>
       </x:c>
       <x:c r="I387" s="11" t="str">
-        <x:v>glm/6152.json</x:v>
+        <x:v>faulty/glm/6152.json</x:v>
       </x:c>
       <x:c r="J387" s="10" t="n">
         <x:f>COUNTA(G387:I387)</x:f>
@@ -16755,13 +16755,13 @@
         <x:v>../references/sps_references_export.ris#record-739</x:v>
       </x:c>
       <x:c r="G391" s="11" t="str">
-        <x:v>deepseek/6248.json</x:v>
+        <x:v>faulty/deepseek/6248.json</x:v>
       </x:c>
       <x:c r="H391" s="11" t="str">
-        <x:v>nemotron/6248.json</x:v>
+        <x:v>faulty/nemotron/6248.json</x:v>
       </x:c>
       <x:c r="I391" s="11" t="str">
-        <x:v>glm/6248.json</x:v>
+        <x:v>faulty/glm/6248.json</x:v>
       </x:c>
       <x:c r="J391" s="10" t="n">
         <x:f>COUNTA(G391:I391)</x:f>
@@ -17128,13 +17128,13 @@
         <x:v>../references/sps_references_export.ris#record-753</x:v>
       </x:c>
       <x:c r="G400" s="11" t="str">
-        <x:v>deepseek/6465.json</x:v>
+        <x:v>faulty/deepseek/6465.json</x:v>
       </x:c>
       <x:c r="H400" s="11" t="str">
-        <x:v>nemotron/6465.json</x:v>
+        <x:v>faulty/nemotron/6465.json</x:v>
       </x:c>
       <x:c r="I400" s="11" t="str">
-        <x:v>glm/6465.json</x:v>
+        <x:v>faulty/glm/6465.json</x:v>
       </x:c>
       <x:c r="J400" s="10" t="n">
         <x:f>COUNTA(G400:I400)</x:f>
@@ -17460,13 +17460,13 @@
         <x:v>../references/sps_references_export.ris#record-768</x:v>
       </x:c>
       <x:c r="G408" s="11" t="str">
-        <x:v>deepseek/6683.json</x:v>
+        <x:v>faulty/deepseek/6683.json</x:v>
       </x:c>
       <x:c r="H408" s="11" t="str">
-        <x:v>nemotron/6683.json</x:v>
+        <x:v>faulty/nemotron/6683.json</x:v>
       </x:c>
       <x:c r="I408" s="11" t="str">
-        <x:v>glm/6683.json</x:v>
+        <x:v>faulty/glm/6683.json</x:v>
       </x:c>
       <x:c r="J408" s="10" t="n">
         <x:f>COUNTA(G408:I408)</x:f>
@@ -18298,13 +18298,13 @@
         <x:v>../references/sps_references_export.ris#record-821</x:v>
       </x:c>
       <x:c r="G428" s="11" t="str">
-        <x:v>deepseek/9111.json</x:v>
+        <x:v>faulty/deepseek/9111.json</x:v>
       </x:c>
       <x:c r="H428" s="11" t="str">
-        <x:v>nemotron/9111.json</x:v>
+        <x:v>faulty/nemotron/9111.json</x:v>
       </x:c>
       <x:c r="I428" s="11" t="str">
-        <x:v>glm/9111.json</x:v>
+        <x:v>faulty/glm/9111.json</x:v>
       </x:c>
       <x:c r="J428" s="10" t="n">
         <x:f>COUNTA(G428:I428)</x:f>
@@ -18339,13 +18339,13 @@
         <x:v>../references/sps_references_export.ris#record-822</x:v>
       </x:c>
       <x:c r="G429" s="11" t="str">
-        <x:v>deepseek/9182.json</x:v>
+        <x:v>faulty/deepseek/9182.json</x:v>
       </x:c>
       <x:c r="H429" s="11" t="str">
-        <x:v>nemotron/9182.json</x:v>
+        <x:v>faulty/nemotron/9182.json</x:v>
       </x:c>
       <x:c r="I429" s="11" t="str">
-        <x:v>glm/9182.json</x:v>
+        <x:v>faulty/glm/9182.json</x:v>
       </x:c>
       <x:c r="J429" s="10" t="n">
         <x:f>COUNTA(G429:I429)</x:f>
@@ -18423,13 +18423,13 @@
         <x:v>../references/sps_references_export.ris#record-825</x:v>
       </x:c>
       <x:c r="G431" s="11" t="str">
-        <x:v>deepseek/9477.json</x:v>
+        <x:v>faulty/deepseek/9477.json</x:v>
       </x:c>
       <x:c r="H431" s="11" t="str">
-        <x:v>nemotron/9477.json</x:v>
+        <x:v>faulty/nemotron/9477.json</x:v>
       </x:c>
       <x:c r="I431" s="11" t="str">
-        <x:v>glm/9477.json</x:v>
+        <x:v>faulty/glm/9477.json</x:v>
       </x:c>
       <x:c r="J431" s="10" t="n">
         <x:f>COUNTA(G431:I431)</x:f>
@@ -18591,13 +18591,13 @@
         <x:v>../references/sps_references_export.ris#record-831</x:v>
       </x:c>
       <x:c r="G435" s="11" t="str">
-        <x:v>deepseek/10691.json</x:v>
+        <x:v>faulty/deepseek/10691.json</x:v>
       </x:c>
       <x:c r="H435" s="11" t="str">
-        <x:v>nemotron/10691.json</x:v>
+        <x:v>faulty/nemotron/10691.json</x:v>
       </x:c>
       <x:c r="I435" s="11" t="str">
-        <x:v>glm/10691.json</x:v>
+        <x:v>faulty/glm/10691.json</x:v>
       </x:c>
       <x:c r="J435" s="10" t="n">
         <x:f>COUNTA(G435:I435)</x:f>
@@ -18761,13 +18761,13 @@
         <x:v>../references/sps_references_export.ris#record-843</x:v>
       </x:c>
       <x:c r="G439" s="11" t="str">
-        <x:v>deepseek/11750.json</x:v>
+        <x:v>faulty/deepseek/11750.json</x:v>
       </x:c>
       <x:c r="H439" s="11" t="str">
-        <x:v>nemotron/11750.json</x:v>
+        <x:v>faulty/nemotron/11750.json</x:v>
       </x:c>
       <x:c r="I439" s="11" t="str">
-        <x:v>glm/11750.json</x:v>
+        <x:v>faulty/glm/11750.json</x:v>
       </x:c>
       <x:c r="J439" s="10" t="n">
         <x:f>COUNTA(G439:I439)</x:f>
@@ -19017,13 +19017,13 @@
         <x:v>../references/sps_references_export.ris#record-852</x:v>
       </x:c>
       <x:c r="G445" s="11" t="str">
-        <x:v>deepseek/11814.json</x:v>
+        <x:v>faulty/deepseek/11814.json</x:v>
       </x:c>
       <x:c r="H445" s="11" t="str">
-        <x:v>nemotron/11814.json</x:v>
+        <x:v>faulty/nemotron/11814.json</x:v>
       </x:c>
       <x:c r="I445" s="11" t="str">
-        <x:v>glm/11814.json</x:v>
+        <x:v>faulty/glm/11814.json</x:v>
       </x:c>
       <x:c r="J445" s="10" t="n">
         <x:f>COUNTA(G445:I445)</x:f>
@@ -19447,13 +19447,13 @@
         <x:v>../references/sps_references_export.ris#record-870</x:v>
       </x:c>
       <x:c r="G455" s="11" t="str">
-        <x:v>deepseek/11928.json</x:v>
+        <x:v>faulty/deepseek/11928.json</x:v>
       </x:c>
       <x:c r="H455" s="11" t="str">
-        <x:v>nemotron/11928.json</x:v>
+        <x:v>faulty/nemotron/11928.json</x:v>
       </x:c>
       <x:c r="I455" s="11" t="str">
-        <x:v>glm/11928.json</x:v>
+        <x:v>faulty/glm/11928.json</x:v>
       </x:c>
       <x:c r="J455" s="10" t="n">
         <x:f>COUNTA(G455:I455)</x:f>
@@ -19576,13 +19576,13 @@
         <x:v>../references/sps_references_export.ris#record-875</x:v>
       </x:c>
       <x:c r="G458" s="11" t="str">
-        <x:v>deepseek/11937.json</x:v>
+        <x:v>faulty/deepseek/11937.json</x:v>
       </x:c>
       <x:c r="H458" s="11" t="str">
-        <x:v>nemotron/11937.json</x:v>
+        <x:v>faulty/nemotron/11937.json</x:v>
       </x:c>
       <x:c r="I458" s="11" t="str">
-        <x:v>glm/11937.json</x:v>
+        <x:v>faulty/glm/11937.json</x:v>
       </x:c>
       <x:c r="J458" s="10" t="n">
         <x:f>COUNTA(G458:I458)</x:f>
@@ -20434,13 +20434,13 @@
         <x:v>../references/sps_references_export.ris#record-911</x:v>
       </x:c>
       <x:c r="G478" s="11" t="str">
-        <x:v>deepseek/12141.json</x:v>
+        <x:v>faulty/deepseek/12141.json</x:v>
       </x:c>
       <x:c r="H478" s="11" t="str">
-        <x:v>nemotron/12141.json</x:v>
+        <x:v>faulty/nemotron/12141.json</x:v>
       </x:c>
       <x:c r="I478" s="11" t="str">
-        <x:v>glm/12141.json</x:v>
+        <x:v>faulty/glm/12141.json</x:v>
       </x:c>
       <x:c r="J478" s="10" t="n">
         <x:f>COUNTA(G478:I478)</x:f>
@@ -20692,13 +20692,13 @@
         <x:v>../references/sps_references_export.ris#record-918</x:v>
       </x:c>
       <x:c r="G484" s="11" t="str">
-        <x:v>deepseek/12244.json</x:v>
+        <x:v>faulty/deepseek/12244.json</x:v>
       </x:c>
       <x:c r="H484" s="11" t="str">
-        <x:v>nemotron/12244.json</x:v>
+        <x:v>faulty/nemotron/12244.json</x:v>
       </x:c>
       <x:c r="I484" s="11" t="str">
-        <x:v>glm/12244.json</x:v>
+        <x:v>faulty/glm/12244.json</x:v>
       </x:c>
       <x:c r="J484" s="10" t="n">
         <x:f>COUNTA(G484:I484)</x:f>
@@ -20735,13 +20735,13 @@
         <x:v>../references/sps_references_export.ris#record-926</x:v>
       </x:c>
       <x:c r="G485" s="11" t="str">
-        <x:v>deepseek/12302.json</x:v>
+        <x:v>faulty/deepseek/12302.json</x:v>
       </x:c>
       <x:c r="H485" s="11" t="str">
-        <x:v>nemotron/12302.json</x:v>
+        <x:v>faulty/nemotron/12302.json</x:v>
       </x:c>
       <x:c r="I485" s="11" t="str">
-        <x:v>glm/12302.json</x:v>
+        <x:v>faulty/glm/12302.json</x:v>
       </x:c>
       <x:c r="J485" s="10" t="n">
         <x:f>COUNTA(G485:I485)</x:f>
@@ -21282,13 +21282,13 @@
         <x:v>../references/sps_references_export.ris#record-976</x:v>
       </x:c>
       <x:c r="G498" s="11" t="str">
-        <x:v>deepseek/12663.json</x:v>
+        <x:v>faulty/deepseek/12663.json</x:v>
       </x:c>
       <x:c r="H498" s="11" t="str">
-        <x:v>nemotron/12663.json</x:v>
+        <x:v>faulty/nemotron/12663.json</x:v>
       </x:c>
       <x:c r="I498" s="11" t="str">
-        <x:v>glm/12663.json</x:v>
+        <x:v>faulty/glm/12663.json</x:v>
       </x:c>
       <x:c r="J498" s="10" t="n">
         <x:f>COUNTA(G498:I498)</x:f>
@@ -21368,13 +21368,13 @@
         <x:v>../references/sps_references_export.ris#record-990</x:v>
       </x:c>
       <x:c r="G500" s="11" t="str">
-        <x:v>deepseek/12751.json</x:v>
+        <x:v>faulty/deepseek/12751.json</x:v>
       </x:c>
       <x:c r="H500" s="11" t="str">
-        <x:v>nemotron/12751.json</x:v>
+        <x:v>faulty/nemotron/12751.json</x:v>
       </x:c>
       <x:c r="I500" s="11" t="str">
-        <x:v>glm/12751.json</x:v>
+        <x:v>faulty/glm/12751.json</x:v>
       </x:c>
       <x:c r="J500" s="10" t="n">
         <x:f>COUNTA(G500:I500)</x:f>
@@ -21624,13 +21624,13 @@
         <x:v>../references/sps_references_export.ris#record-1011</x:v>
       </x:c>
       <x:c r="G506" s="11" t="str">
-        <x:v>deepseek/13049.json</x:v>
+        <x:v>faulty/deepseek/13049.json</x:v>
       </x:c>
       <x:c r="H506" s="11" t="str">
-        <x:v>nemotron/13049.json</x:v>
+        <x:v>faulty/nemotron/13049.json</x:v>
       </x:c>
       <x:c r="I506" s="11" t="str">
-        <x:v>glm/13049.json</x:v>
+        <x:v>faulty/glm/13049.json</x:v>
       </x:c>
       <x:c r="J506" s="10" t="n">
         <x:f>COUNTA(G506:I506)</x:f>
@@ -21667,13 +21667,13 @@
         <x:v>../references/sps_references_export.ris#record-1014</x:v>
       </x:c>
       <x:c r="G507" s="11" t="str">
-        <x:v>deepseek/13066.json</x:v>
+        <x:v>faulty/deepseek/13066.json</x:v>
       </x:c>
       <x:c r="H507" s="11" t="str">
-        <x:v>nemotron/13066.json</x:v>
+        <x:v>faulty/nemotron/13066.json</x:v>
       </x:c>
       <x:c r="I507" s="11" t="str">
-        <x:v>glm/13066.json</x:v>
+        <x:v>faulty/glm/13066.json</x:v>
       </x:c>
       <x:c r="J507" s="10" t="n">
         <x:f>COUNTA(G507:I507)</x:f>
@@ -21966,13 +21966,13 @@
         <x:v>../references/sps_references_export.ris#record-1039</x:v>
       </x:c>
       <x:c r="G514" s="11" t="str">
-        <x:v>deepseek/13804.json</x:v>
+        <x:v>faulty/deepseek/13804.json</x:v>
       </x:c>
       <x:c r="H514" s="11" t="str">
-        <x:v>nemotron/13804.json</x:v>
+        <x:v>faulty/nemotron/13804.json</x:v>
       </x:c>
       <x:c r="I514" s="11" t="str">
-        <x:v>glm/13804.json</x:v>
+        <x:v>faulty/glm/13804.json</x:v>
       </x:c>
       <x:c r="J514" s="10" t="n">
         <x:f>COUNTA(G514:I514)</x:f>
@@ -21992,7 +21992,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53bb1ac049374732"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc476d42ffc2642db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>